<commit_message>
lote: one zip per video instead of two big zips
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Su43BFuF4GRbx64xuEPvfV
</commit_message>
<xml_diff>
--- a/agendamento/lote-01-10/schedule-videos-01-10.xlsx
+++ b/agendamento/lote-01-10/schedule-videos-01-10.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video01/video01.mp4</t>
+          <t>video01.zip › video01/video01.mp4</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video01/short1.mp4</t>
+          <t>video01.zip › video01/short1.mp4</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video01/short2.mp4</t>
+          <t>video01.zip › video01/short2.mp4</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video02/video02.mp4</t>
+          <t>video02.zip › video02/video02.mp4</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video02/short1.mp4</t>
+          <t>video02.zip › video02/short1.mp4</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video02/short2.mp4</t>
+          <t>video02.zip › video02/short2.mp4</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video03/video03.mp4</t>
+          <t>video03.zip › video03/video03.mp4</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video03/short1.mp4</t>
+          <t>video03.zip › video03/short1.mp4</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video03/short2.mp4</t>
+          <t>video03.zip › video03/short2.mp4</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video03/short3.mp4</t>
+          <t>video03.zip › video03/short3.mp4</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video03/short4.mp4</t>
+          <t>video03.zip › video03/short4.mp4</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video04/video04.mp4</t>
+          <t>video04.zip › video04/video04.mp4</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video04/short1.mp4</t>
+          <t>video04.zip › video04/short1.mp4</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video04/short2.mp4</t>
+          <t>video04.zip › video04/short2.mp4</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video04/short3.mp4</t>
+          <t>video04.zip › video04/short3.mp4</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video04/short4.mp4</t>
+          <t>video04.zip › video04/short4.mp4</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video05/video05.mp4</t>
+          <t>video05.zip › video05/video05.mp4</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video05/short1.mp4</t>
+          <t>video05.zip › video05/short1.mp4</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video05/short2.mp4</t>
+          <t>video05.zip › video05/short2.mp4</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video05/short3.mp4</t>
+          <t>video05.zip › video05/short3.mp4</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-01-05.zip › video05/short4.mp4</t>
+          <t>video05.zip › video05/short4.mp4</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video06/video06.mp4</t>
+          <t>video06.zip › video06/video06.mp4</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video06/short1.mp4</t>
+          <t>video06.zip › video06/short1.mp4</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video06/short2.mp4</t>
+          <t>video06.zip › video06/short2.mp4</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video06/short3.mp4</t>
+          <t>video06.zip › video06/short3.mp4</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video06/short4.mp4</t>
+          <t>video06.zip › video06/short4.mp4</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video07/video07.mp4</t>
+          <t>video07.zip › video07/video07.mp4</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video07/short1.mp4</t>
+          <t>video07.zip › video07/short1.mp4</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video07/short2.mp4</t>
+          <t>video07.zip › video07/short2.mp4</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video07/short3.mp4</t>
+          <t>video07.zip › video07/short3.mp4</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video07/short4.mp4</t>
+          <t>video07.zip › video07/short4.mp4</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video08/video08.mp4</t>
+          <t>video08.zip › video08/video08.mp4</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video08/short1.mp4</t>
+          <t>video08.zip › video08/short1.mp4</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video08/short2.mp4</t>
+          <t>video08.zip › video08/short2.mp4</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video08/short3.mp4</t>
+          <t>video08.zip › video08/short3.mp4</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video08/short4.mp4</t>
+          <t>video08.zip › video08/short4.mp4</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video09/video09.mp4</t>
+          <t>video09.zip › video09/video09.mp4</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video09/short1.mp4</t>
+          <t>video09.zip › video09/short1.mp4</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video09/short2.mp4</t>
+          <t>video09.zip › video09/short2.mp4</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video09/short3.mp4</t>
+          <t>video09.zip › video09/short3.mp4</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video09/short4.mp4</t>
+          <t>video09.zip › video09/short4.mp4</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video10/video10.mp4</t>
+          <t>video10.zip › video10/video10.mp4</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video10/short1.mp4</t>
+          <t>video10.zip › video10/short1.mp4</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video10/short2.mp4</t>
+          <t>video10.zip › video10/short2.mp4</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video10/short3.mp4</t>
+          <t>video10.zip › video10/short3.mp4</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>pickup-reality-06-10.zip › video10/short4.mp4</t>
+          <t>video10.zip › video10/short4.mp4</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">

</xml_diff>